<commit_message>
updated research and projects page
</commit_message>
<xml_diff>
--- a/data/news.xlsx
+++ b/data/news.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anwaypimpalkar/everything/anwaypimpalkar.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A0BAFC-76ED-114B-ADD4-064B1151DE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9992C0C3-978A-F848-A185-C98D47D22AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17820" xr2:uid="{46DB94BC-6658-C940-A428-5CA04B255DCE}"/>
+    <workbookView xWindow="-38400" yWindow="-3720" windowWidth="38400" windowHeight="21120" xr2:uid="{46DB94BC-6658-C940-A428-5CA04B255DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="projects" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>year</t>
   </si>
@@ -46,12 +46,6 @@
     <t>Starting my PhD at Harvard Engineering!</t>
   </si>
   <si>
-    <t>July</t>
-  </si>
-  <si>
-    <t>Had an amazing time home in Pune, charged.</t>
-  </si>
-  <si>
     <t>June</t>
   </si>
   <si>
@@ -95,9 +89,6 @@
   </si>
   <si>
     <t>Starting my Master's in BME at Johns Hopkins!</t>
-  </si>
-  <si>
-    <t>unfiltered;</t>
   </si>
   <si>
     <t>body</t>
@@ -1104,14 +1095,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36804C05-0050-DB4A-B44D-23DEA2DFD96A}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.5" style="1" customWidth="1"/>
     <col min="3" max="3" width="68.1640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="71.1640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="40.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="54.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="59.1640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="80.83203125" style="1" customWidth="1"/>
@@ -1132,7 +1123,7 @@
         <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
@@ -1161,10 +1152,10 @@
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="8"/>
@@ -1174,7 +1165,7 @@
       <c r="L2" s="9"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="57" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>2025</v>
       </c>
@@ -1184,34 +1175,35 @@
       <c r="C3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="D3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>35</v>
+      </c>
       <c r="F3" s="7"/>
-      <c r="G3" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="G3" s="7"/>
       <c r="H3" s="8"/>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
       <c r="L3" s="9"/>
-      <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:13" ht="57" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" s="4" customFormat="1" ht="38" x14ac:dyDescent="0.25">
       <c r="A4" s="7">
         <v>2025</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>11</v>
-      </c>
       <c r="D4" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
@@ -1220,22 +1212,23 @@
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
       <c r="L4" s="9"/>
+      <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:13" s="4" customFormat="1" ht="38" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" s="4" customFormat="1" ht="76" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
         <v>2025</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
@@ -1246,22 +1239,20 @@
       <c r="L5" s="9"/>
       <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="1:13" s="4" customFormat="1" ht="76" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>2025</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>14</v>
-      </c>
       <c r="D6" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="E6" s="7"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="8"/>
@@ -1269,22 +1260,23 @@
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
       <c r="L6" s="9"/>
-      <c r="M6" s="1"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="38" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>2025</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="7"/>
+        <v>29</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>38</v>
+      </c>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="8"/>
@@ -1298,16 +1290,16 @@
         <v>2025</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>32</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
@@ -1328,11 +1320,9 @@
         <v>17</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>42</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="8"/>
@@ -1341,9 +1331,9 @@
       <c r="K9" s="7"/>
       <c r="L9" s="9"/>
     </row>
-    <row r="10" spans="1:13" ht="38" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>18</v>
@@ -1351,9 +1341,7 @@
       <c r="C10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>34</v>
-      </c>
+      <c r="D10" s="7"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
@@ -1368,30 +1356,25 @@
         <v>2024</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>2024</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -1400,37 +1383,22 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
-        <v>2023</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-    </row>
-    <row r="19" spans="3:3" ht="20" x14ac:dyDescent="0.25">
-      <c r="C19" s="1" t="s">
-        <v>29</v>
+    <row r="18" spans="3:3" ht="20" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated projects and news
</commit_message>
<xml_diff>
--- a/data/news.xlsx
+++ b/data/news.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anwaypimpalkar/everything/anwaypimpalkar.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E411CA5-5B00-7740-A273-7A9AA0370E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87558CD-761D-E142-AD90-BCA9282D6FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{46DB94BC-6658-C940-A428-5CA04B255DCE}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
   <si>
     <t>year</t>
   </si>
@@ -97,9 +97,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>Grateful to be part of this vibrant community of scholars and engineers.</t>
-  </si>
-  <si>
     <t>Had the chance to share my work on optimizing multimodal feedback at RehabWeek in Chicago. Grateful for the opportunity to present to such a clinically impact-driven audience, and for the really insightful conversations throughout.</t>
   </si>
   <si>
@@ -112,9 +109,6 @@
     <t>Thrilled to be selected for the NDSEG Fellowship, supporting three years of my tuition and stipend towards my PhD!</t>
   </si>
   <si>
-    <t>Two down, one to go!</t>
-  </si>
-  <si>
     <t>/assets/images/news/Harvard_SEC.jpg</t>
   </si>
   <si>
@@ -130,10 +124,13 @@
     <t>/assets/images/news/NDSEG.png</t>
   </si>
   <si>
-    <t>Excited to be able to join Prof. Katia Bertoldi and Prof. Giovanni Traverso for this marathon.</t>
-  </si>
-  <si>
     <t>Helped organize the first Hopkins-India Conference in Washington DC!</t>
+  </si>
+  <si>
+    <t>Grateful to be a part of a vibrant community of scholars and engineers supported through industry partnerships, professional development, and a strong national network.</t>
+  </si>
+  <si>
+    <t>Two down, one more to go!</t>
   </si>
 </sst>
 </file>
@@ -1144,11 +1141,9 @@
       <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>36</v>
-      </c>
+      <c r="D2" s="7"/>
       <c r="E2" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>23</v>
@@ -1161,7 +1156,7 @@
       <c r="L2" s="9"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" s="4" customFormat="1" ht="38" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" s="4" customFormat="1" ht="57" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>2025</v>
       </c>
@@ -1172,10 +1167,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
@@ -1197,10 +1192,10 @@
         <v>11</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
@@ -1222,7 +1217,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
@@ -1241,13 +1236,13 @@
         <v>10</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
@@ -1268,10 +1263,10 @@
         <v>14</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -1292,7 +1287,7 @@
         <v>16</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>

</xml_diff>